<commit_message>
CI: Auto Update Data
</commit_message>
<xml_diff>
--- a/Excel/悖论&模组作业作者版.xlsx
+++ b/Excel/悖论&模组作业作者版.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>maa://25390 (95.47), maa://24702 (94.84), maa://36681 (86.42)</t>
+          <t>maa://25390 (95.48), maa://24702 (94.84), maa://36681 (86.42)</t>
         </is>
       </c>
       <c r="E2" s="11" t="n"/>
@@ -725,12 +725,12 @@
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L2" s="14" t="inlineStr">
         <is>
-          <t>maa://39402 (94.87), *maa://30515 (70.37), *maa://34787 (73.91)</t>
+          <t>maa://39402 (94.87), *maa://34787 (73.91)</t>
         </is>
       </c>
       <c r="M2" s="11" t="n"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>maa://40192 (96.23), maa://36987 (96.23), maa://39849 (88.89)</t>
+          <t>maa://40192 (96.26), maa://36987 (96.23), maa://39849 (88.89)</t>
         </is>
       </c>
       <c r="E3" s="11" t="n"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="H3" s="14" t="inlineStr">
         <is>
-          <t>maa://21247 (98.46)</t>
+          <t>maa://21247 (98.47)</t>
         </is>
       </c>
       <c r="I3" s="11" t="n"/>
@@ -860,7 +860,7 @@
       </c>
       <c r="L3" s="14" t="inlineStr">
         <is>
-          <t>*maa://22880 (65.95), maa://20276 (88.63), *maa://22749 (77.78)</t>
+          <t>*maa://22880 (66.24), maa://20276 (88.63), *maa://22749 (77.78)</t>
         </is>
       </c>
       <c r="M3" s="11" t="n"/>
@@ -924,7 +924,7 @@
       </c>
       <c r="AB3" s="14" t="inlineStr">
         <is>
-          <t>maa://24390 (95.6), maa://52241 (100.0)</t>
+          <t>maa://24390 (95.65), maa://52241 (100.0)</t>
         </is>
       </c>
       <c r="AC3" s="11" t="n"/>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>maa://32509 (93.98), maa://27295 (88.3), maa://22754 (89.19), *maa://31008 (79.55)</t>
+          <t>maa://32509 (93.98), maa://27295 (88.42), maa://22754 (89.19), *maa://31008 (79.55)</t>
         </is>
       </c>
       <c r="U4" s="11" t="n"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>maa://21245 (84.56), maa://22744 (82.14), maa://54105 (100.0)</t>
+          <t>maa://21245 (84.62), maa://22744 (82.14), maa://54105 (100.0)</t>
         </is>
       </c>
       <c r="E5" s="11" t="n"/>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>maa://24839 (98.83)</t>
+          <t>maa://24839 (98.84)</t>
         </is>
       </c>
       <c r="M6" s="11" t="n"/>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="X6" s="14" t="inlineStr">
         <is>
-          <t>maa://52754 (82.35)</t>
+          <t>maa://52754 (83.33)</t>
         </is>
       </c>
       <c r="Y6" s="11" t="n"/>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>maa://28624 (93.84), maa://24957 (97.78)</t>
+          <t>maa://28624 (93.88), maa://24957 (97.78)</t>
         </is>
       </c>
       <c r="M7" s="11" t="n"/>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>maa://21291 (86.67)</t>
+          <t>maa://21291 (87.1)</t>
         </is>
       </c>
       <c r="U7" s="11" t="n"/>
@@ -1473,7 +1473,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>更新日期：2025.06.14 13:21:08</t>
+          <t>更新日期：2025.06.15 13:20:11</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>*maa://24371 (55.13)</t>
+          <t>*maa://24371 (55.7)</t>
         </is>
       </c>
       <c r="I8" s="11" t="n"/>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="P9" s="14" t="inlineStr">
         <is>
-          <t>maa://22736 (83.33)</t>
+          <t>maa://22736 (83.48)</t>
         </is>
       </c>
       <c r="Q9" s="11" t="n"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="T9" s="14" t="inlineStr">
         <is>
-          <t>maa://26222 (98.33)</t>
+          <t>maa://26222 (98.36)</t>
         </is>
       </c>
       <c r="U9" s="11" t="n"/>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="AB9" s="14" t="inlineStr">
         <is>
-          <t>maa://28711 (87.32), maa://40166 (93.88)</t>
+          <t>maa://28711 (87.41), maa://40166 (93.88)</t>
         </is>
       </c>
       <c r="AC9" s="11" t="n"/>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="AF9" s="14" t="inlineStr">
         <is>
-          <t>maa://26206 (89.27), *maa://22865 (53.57)</t>
+          <t>maa://26206 (89.33), *maa://22865 (53.57)</t>
         </is>
       </c>
       <c r="AG9" s="27" t="n"/>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>***maa://25695 (18.72), ***maa://39951 (11.84), ***maa://34206 (22.22), *maa://45271 (60.76), ***maa://39243 (25.0), **maa://54000 (33.33)</t>
+          <t>***maa://25695 (18.63), ***maa://39951 (11.84), ***maa://34206 (22.22), *maa://45271 (61.73), ***maa://39243 (25.0), **maa://54000 (33.33)</t>
         </is>
       </c>
       <c r="E10" s="11" t="n"/>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="T10" s="14" t="inlineStr">
         <is>
-          <t>maa://27395 (96.75), maa://22755 (89.15)</t>
+          <t>maa://27395 (96.76), maa://22755 (89.15)</t>
         </is>
       </c>
       <c r="U10" s="11" t="n"/>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="X10" s="14" t="inlineStr">
         <is>
-          <t>maa://22301 (97.91), maa://45828 (93.48), maa://22726 (100.0)</t>
+          <t>maa://22301 (97.93), maa://45828 (93.48), maa://22726 (100.0)</t>
         </is>
       </c>
       <c r="Y10" s="11" t="n"/>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="AF10" s="14" t="inlineStr">
         <is>
-          <t>*maa://25021 (54.21), *maa://22733 (64.29), **maa://22761 (50.0)</t>
+          <t>*maa://25021 (53.7), *maa://22733 (64.29), **maa://22761 (50.0)</t>
         </is>
       </c>
       <c r="AG10" s="27" t="n"/>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="X12" s="14" t="inlineStr">
         <is>
-          <t>maa://22753 (91.94), *maa://21485 (75.84), maa://37962 (92.65)</t>
+          <t>maa://22753 (91.98), *maa://21485 (75.84), maa://37962 (92.75)</t>
         </is>
       </c>
       <c r="Y12" s="11" t="n"/>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="AB12" s="14" t="inlineStr">
         <is>
-          <t>maa://23669 (95.67), maa://36677 (95.35), maa://39872 (93.1)</t>
+          <t>maa://23669 (95.68), maa://36677 (95.35), maa://39872 (93.1)</t>
         </is>
       </c>
       <c r="AC12" s="11" t="n"/>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>maa://24999 (92.74), maa://36673 (91.95), maa://25001 (86.49)</t>
+          <t>maa://24999 (92.75), maa://36673 (91.95), maa://25001 (86.49)</t>
         </is>
       </c>
       <c r="E13" s="11" t="n"/>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>maa://30764 (89.86)</t>
+          <t>maa://30764 (90.0)</t>
         </is>
       </c>
       <c r="E14" s="11" t="n"/>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>maa://39841 (94.41), maa://26245 (96.72), maa://21288 (96.3), maa://36682 (95.92)</t>
+          <t>maa://39841 (94.44), maa://26245 (96.72), maa://21288 (96.3), maa://36682 (95.92)</t>
         </is>
       </c>
       <c r="M14" s="11" t="n"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="P14" s="14" t="inlineStr">
         <is>
-          <t>maa://23250 (98.87), maa://20107 (87.1), maa://22772 (100.0)</t>
+          <t>maa://23250 (98.88), maa://20107 (87.1), maa://22772 (100.0)</t>
         </is>
       </c>
       <c r="Q14" s="11" t="n"/>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="T14" s="14" t="inlineStr">
         <is>
-          <t>maa://22521 (94.87), maa://42751 (100.0)</t>
+          <t>maa://22521 (94.92), maa://42751 (100.0)</t>
         </is>
       </c>
       <c r="U14" s="11" t="n"/>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="X14" s="14" t="inlineStr">
         <is>
-          <t>maa://37468 (92.0)</t>
+          <t>maa://37468 (92.31)</t>
         </is>
       </c>
       <c r="Y14" s="11" t="n"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>maa://24304 (87.06), maa://21478 (90.0)</t>
+          <t>maa://24304 (87.16), maa://21478 (90.0)</t>
         </is>
       </c>
       <c r="I15" s="11" t="n"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="P15" s="14" t="inlineStr">
         <is>
-          <t>maa://24762 (91.35), *maa://22727 (70.0)</t>
+          <t>maa://24762 (91.4), *maa://22727 (70.0)</t>
         </is>
       </c>
       <c r="Q15" s="11" t="n"/>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="T15" s="14" t="inlineStr">
         <is>
-          <t>maa://23892 (96.63)</t>
+          <t>maa://23892 (96.67)</t>
         </is>
       </c>
       <c r="U15" s="11" t="n"/>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>maa://22430 (89.67), maa://39599 (86.75)</t>
+          <t>maa://22430 (89.72), maa://39599 (86.9)</t>
         </is>
       </c>
       <c r="I17" s="11" t="n"/>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="AF17" s="14" t="inlineStr">
         <is>
-          <t>maa://50136 (95.45)</t>
+          <t>maa://50136 (95.83)</t>
         </is>
       </c>
       <c r="AG17" s="27" t="n"/>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>maa://24570 (97.07)</t>
+          <t>maa://24570 (97.08)</t>
         </is>
       </c>
       <c r="E18" s="11" t="n"/>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="L18" s="14" t="inlineStr">
         <is>
-          <t>maa://22466 (92.12), maa://52226 (95.65)</t>
+          <t>maa://22466 (92.16), maa://52226 (95.65)</t>
         </is>
       </c>
       <c r="M18" s="11" t="n"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="AB19" s="14" t="inlineStr">
         <is>
-          <t>*maa://30709 (68.66), *maa://36668 (57.32)</t>
+          <t>*maa://30709 (68.79), *maa://36668 (57.32)</t>
         </is>
       </c>
       <c r="AC19" s="11" t="n"/>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>maa://22864 (90.86)</t>
+          <t>maa://22864 (90.37)</t>
         </is>
       </c>
       <c r="I20" s="11" t="n"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="L20" s="14" t="inlineStr">
         <is>
-          <t>maa://41331 (86.17)</t>
+          <t>maa://41331 (86.27)</t>
         </is>
       </c>
       <c r="M20" s="11" t="n"/>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="P20" s="14" t="inlineStr">
         <is>
-          <t>maa://37442 (96.15)</t>
+          <t>maa://37442 (96.23)</t>
         </is>
       </c>
       <c r="Q20" s="11" t="n"/>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="X20" s="14" t="inlineStr">
         <is>
-          <t>maa://50085 (88.03), maa://49976 (86.59), maa://56241 (88.89)</t>
+          <t>maa://50085 (88.28), maa://49976 (86.59), maa://56241 (88.89)</t>
         </is>
       </c>
       <c r="Y20" s="11" t="n"/>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>maa://21261 (98.0)</t>
+          <t>maa://21261 (98.04)</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>maa://24372 (97.17)</t>
+          <t>maa://24372 (97.2)</t>
         </is>
       </c>
       <c r="I21" s="11" t="n"/>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="AB21" s="14" t="inlineStr">
         <is>
-          <t>maa://21443 (82.81), ***maa://23820 (30.0), **maa://52223 (40.62)</t>
+          <t>maa://21443 (82.81), ***maa://23820 (30.0), **maa://52223 (39.39)</t>
         </is>
       </c>
       <c r="AC21" s="11" t="n"/>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="X22" s="14" t="inlineStr">
         <is>
-          <t>maa://21282 (98.72), *maa://37649 (73.81)</t>
+          <t>maa://21282 (98.73), *maa://37649 (73.81)</t>
         </is>
       </c>
       <c r="Y22" s="11" t="n"/>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="P23" s="14" t="inlineStr">
         <is>
-          <t>maa://30587 (92.09), *maa://29748 (76.3), *maa://37566 (78.26)</t>
+          <t>maa://30587 (92.13), *maa://29748 (76.3), *maa://37566 (78.26)</t>
         </is>
       </c>
       <c r="Q23" s="11" t="n"/>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="T23" s="14" t="inlineStr">
         <is>
-          <t>maa://31212 (89.47), maa://24387 (82.93)</t>
+          <t>maa://31212 (89.74), maa://24387 (82.93)</t>
         </is>
       </c>
       <c r="U23" s="11" t="n"/>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="X24" s="14" t="inlineStr">
         <is>
-          <t>maa://29988 (84.92), maa://23504 (93.7), *maa://25141 (77.37), *maa://36663 (78.0), maa://52227 (100.0)</t>
+          <t>maa://29988 (84.92), maa://23504 (93.71), *maa://25141 (77.37), *maa://36663 (78.0), maa://52227 (100.0)</t>
         </is>
       </c>
       <c r="Y24" s="11" t="n"/>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="AF24" s="14" t="inlineStr">
         <is>
-          <t>maa://22523 (81.74), *maa://36672 (75.76), maa://29910 (93.75), maa://45831 (86.67)</t>
+          <t>maa://22523 (81.74), *maa://36672 (74.63), maa://29910 (93.85), maa://45831 (87.5)</t>
         </is>
       </c>
       <c r="AG24" s="27" t="n"/>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>maa://29753 (95.47)</t>
+          <t>maa://29753 (95.48)</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="AB25" s="14" t="inlineStr">
         <is>
-          <t>maa://31215 (89.51), *maa://24516 (79.57), maa://26001 (84.75)</t>
+          <t>maa://31215 (89.66), *maa://24516 (79.57), maa://26001 (84.75)</t>
         </is>
       </c>
       <c r="AC25" s="11" t="n"/>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="AF25" s="14" t="inlineStr">
         <is>
-          <t>maa://20108 (95.89), maa://24621 (97.18), maa://36676 (97.06), maa://22771 (85.71), *maa://37772 (80.0)</t>
+          <t>maa://20108 (95.92), maa://24621 (97.18), maa://36676 (97.06), maa://22771 (85.71), *maa://37772 (80.0)</t>
         </is>
       </c>
       <c r="AG25" s="27" t="n"/>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="AB26" s="14" t="inlineStr">
         <is>
-          <t>maa://42235 (96.05)</t>
+          <t>maa://42235 (96.08)</t>
         </is>
       </c>
       <c r="AC26" s="11" t="n"/>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="AF26" s="14" t="inlineStr">
         <is>
-          <t>*maa://30511 (75.0), *maa://29760 (52.94)</t>
+          <t>*maa://30511 (75.47), *maa://29760 (52.94)</t>
         </is>
       </c>
       <c r="AG26" s="27" t="n"/>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>*maa://39601 (79.17), maa://34494 (97.3)</t>
+          <t>maa://39601 (80.77), maa://34494 (97.3)</t>
         </is>
       </c>
       <c r="I27" s="11" t="n"/>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="AF27" s="14" t="inlineStr">
         <is>
-          <t>maa://24023 (96.15)</t>
+          <t>maa://24023 (96.2)</t>
         </is>
       </c>
       <c r="AG27" s="27" t="n"/>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="X28" s="14" t="inlineStr">
         <is>
-          <t>maa://39929 (91.97), maa://41749 (92.25)</t>
+          <t>maa://39929 (91.97), maa://41749 (92.31)</t>
         </is>
       </c>
       <c r="Y28" s="11" t="n"/>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="AF28" s="14" t="inlineStr">
         <is>
-          <t>maa://36660 (92.54)</t>
+          <t>maa://36660 (92.58)</t>
         </is>
       </c>
       <c r="AG28" s="27" t="n"/>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>maa://28432 (94.05), maa://31400 (98.89), maa://28440 (83.94), *maa://28650 (71.43)</t>
+          <t>maa://28432 (94.05), maa://31400 (98.89), maa://28440 (84.06), *maa://28650 (71.43)</t>
         </is>
       </c>
       <c r="M29" s="11" t="n"/>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>maa://45792 (89.66)</t>
+          <t>maa://45792 (90.0)</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -4510,7 +4510,7 @@
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>maa://35926 (93.75), maa://36258 (87.88), *maa://43904 (73.33)</t>
+          <t>maa://35926 (93.75), maa://36258 (87.95), *maa://43904 (73.33)</t>
         </is>
       </c>
       <c r="M31" s="11" t="n"/>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>maa://21895 (97.63), maa://36667 (97.32), maa://22760 (100.0)</t>
+          <t>maa://21895 (97.64), maa://36667 (97.32), maa://22760 (100.0)</t>
         </is>
       </c>
       <c r="I32" s="11" t="n"/>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="T32" s="14" t="inlineStr">
         <is>
-          <t>maa://42859 (96.98), maa://41108 (86.27), maa://41238 (97.99), maa://45523 (100.0)</t>
+          <t>maa://42859 (97.0), maa://41108 (86.27), maa://41238 (97.99), maa://45523 (100.0)</t>
         </is>
       </c>
       <c r="U32" s="11" t="n"/>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="P34" s="14" t="inlineStr">
         <is>
-          <t>maa://48817 (96.88), maa://56235 (100.0)</t>
+          <t>maa://48817 (96.92), maa://56235 (100.0)</t>
         </is>
       </c>
       <c r="Q34" s="11" t="n"/>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>maa://24375 (90.7)</t>
+          <t>maa://24375 (90.91)</t>
         </is>
       </c>
       <c r="I36" s="11" t="n"/>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="AF38" s="14" t="inlineStr">
         <is>
-          <t>maa://36697 (89.31)</t>
+          <t>maa://36697 (89.34)</t>
         </is>
       </c>
       <c r="AG38" s="27" t="n"/>
@@ -5460,7 +5460,7 @@
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>maa://36670 (89.57), maa://25199 (85.22), maa://30434 (93.13), *maa://45059 (79.41)</t>
+          <t>maa://36670 (89.57), maa://25199 (85.22), maa://30434 (93.18), *maa://45059 (79.41)</t>
         </is>
       </c>
       <c r="I39" s="11" t="n"/>
@@ -5662,7 +5662,7 @@
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>maa://24466 (93.88)</t>
+          <t>maa://24466 (94.0)</t>
         </is>
       </c>
       <c r="I41" s="11" t="n"/>
@@ -5986,7 +5986,7 @@
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>maa://21229 (84.42), maa://30807 (93.51), maa://42459 (89.47)</t>
+          <t>maa://21229 (84.42), maa://30807 (93.51), maa://42459 (87.18)</t>
         </is>
       </c>
       <c r="I45" s="11" t="n"/>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>maa://35931 (92.67), maa://43901 (94.74)</t>
+          <t>maa://35931 (92.71), maa://43901 (94.74)</t>
         </is>
       </c>
       <c r="I46" s="11" t="n"/>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="P52" s="14" t="inlineStr">
         <is>
-          <t>maa://59378 (96.88), maa://59394 (91.67)</t>
+          <t>maa://59378 (96.88), maa://59394 (93.33)</t>
         </is>
       </c>
       <c r="Q52" s="11" t="n"/>
@@ -6433,7 +6433,7 @@
       </c>
       <c r="H53" s="14" t="inlineStr">
         <is>
-          <t>maa://32534 (95.13)</t>
+          <t>maa://32534 (95.15)</t>
         </is>
       </c>
       <c r="I53" s="11" t="n"/>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>*maa://40438 (74.68)</t>
+          <t>*maa://40438 (75.0)</t>
         </is>
       </c>
       <c r="I60" s="11" t="n"/>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>maa://59534 (97.5), maa://59413 (100.0)</t>
+          <t>maa://59534 (97.62), maa://59413 (100.0)</t>
         </is>
       </c>
       <c r="I63" s="11" t="n"/>
@@ -6958,7 +6958,7 @@
     <row r="1" ht="13.5" customFormat="1" customHeight="1" s="17">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>更新日期：2025.06.14 13:21:08</t>
+          <t>更新日期：2025.06.15 13:20:11</t>
         </is>
       </c>
       <c r="E1" s="16" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="D32" s="20" t="inlineStr">
         <is>
-          <t>maa://36644 (88.42), maa://36866 (96.15), maa://45572 (91.67), maa://27794 (100.0), maa://20960 (100.0), maa://20843 (100.0), **maa://24483 (50.0), maa://20862 (83.33), *maa://20893 (77.78)</t>
+          <t>maa://36644 (88.42), maa://36866 (96.23), maa://45572 (91.67), maa://27794 (100.0), maa://20960 (100.0), maa://20843 (100.0), **maa://24483 (50.0), maa://20862 (83.33), *maa://20893 (77.78)</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="D34" s="20" t="inlineStr">
         <is>
-          <t>maa://20916 (82.86), maa://52658 (87.5)</t>
+          <t>maa://20916 (82.86), maa://52658 (88.89)</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
@@ -12142,7 +12142,7 @@
       </c>
       <c r="D97" s="20" t="inlineStr">
         <is>
-          <t>maa://20991 (100.0), maa://51015 (85.71)</t>
+          <t>maa://20991 (100.0), maa://51015 (86.36)</t>
         </is>
       </c>
       <c r="E97" s="21" t="inlineStr">
@@ -12250,7 +12250,7 @@
       </c>
       <c r="D99" s="20" t="inlineStr">
         <is>
-          <t>maa://20929 (94.74)</t>
+          <t>maa://20929 (95.0)</t>
         </is>
       </c>
       <c r="E99" s="21" t="inlineStr">
@@ -12736,7 +12736,7 @@
       </c>
       <c r="D108" s="20" t="inlineStr">
         <is>
-          <t>maa://25018 (96.63), maa://51881 (99.16), maa://25776 (92.11), maa://28361 (97.37), maa://25772 (94.12), maa://56588 (94.12), maa://45194 (87.5), maa://32653 (85.71), maa://25161 (81.25)</t>
+          <t>maa://25018 (96.64), maa://51881 (99.17), maa://25776 (92.11), maa://28361 (97.37), maa://25772 (94.12), maa://56588 (94.44), maa://45194 (87.5), maa://32653 (85.71), maa://25161 (81.25)</t>
         </is>
       </c>
       <c r="E108" s="21" t="inlineStr">
@@ -13006,7 +13006,7 @@
       </c>
       <c r="D113" s="20" t="inlineStr">
         <is>
-          <t>maa://29037 (98.46)</t>
+          <t>maa://29037 (98.48)</t>
         </is>
       </c>
       <c r="E113" s="21" t="inlineStr">
@@ -13492,7 +13492,7 @@
       </c>
       <c r="D122" s="20" t="inlineStr">
         <is>
-          <t>maa://29650 (98.31), maa://45570 (97.87)</t>
+          <t>maa://29650 (98.31), maa://45570 (97.92)</t>
         </is>
       </c>
       <c r="E122" s="21" t="inlineStr">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="D139" s="20" t="inlineStr">
         <is>
-          <t>**maa://30679 (50.0), maa://45258 (92.86)</t>
+          <t>**maa://30679 (50.0), maa://45258 (93.33)</t>
         </is>
       </c>
       <c r="E139" s="21" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="D143" s="20" t="inlineStr">
         <is>
-          <t>maa://30670 (96.6), maa://31470 (96.67), *maa://45066 (66.67), **maa://30867 (40.0)</t>
+          <t>maa://30670 (96.64), maa://31470 (96.67), *maa://45066 (66.67), **maa://30867 (40.0)</t>
         </is>
       </c>
       <c r="E143" s="21" t="inlineStr">
@@ -14950,7 +14950,7 @@
       </c>
       <c r="D149" s="20" t="inlineStr">
         <is>
-          <t>maa://36641 (98.44), maa://40957 (93.36), maa://36865 (96.32), maa://44635 (87.74), maa://44660 (92.31), maa://41128 (83.78), maa://42918 (100.0), maa://44119 (97.44), maa://46108 (100.0), maa://37300 (100.0), maa://42917 (100.0)</t>
+          <t>maa://36641 (98.44), maa://40957 (93.38), maa://36865 (96.32), maa://44635 (87.74), maa://44660 (92.31), maa://41128 (83.78), maa://42918 (100.0), maa://44119 (97.44), maa://46108 (100.0), maa://37300 (100.0), maa://42917 (100.0)</t>
         </is>
       </c>
       <c r="E149" s="21" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="D150" s="20" t="inlineStr">
         <is>
-          <t>maa://51549 (95.12), maa://51923 (95.65)</t>
+          <t>maa://51549 (95.24), maa://51923 (95.65)</t>
         </is>
       </c>
       <c r="E150" s="21" t="inlineStr">
@@ -17758,7 +17758,7 @@
       </c>
       <c r="D201" s="20" t="inlineStr">
         <is>
-          <t>maa://42223 (99.59), maa://49077 (94.29), maa://42292 (97.22), maa://42402 (100.0)</t>
+          <t>maa://42223 (99.6), maa://49077 (94.29), maa://42292 (97.22), maa://42402 (100.0)</t>
         </is>
       </c>
       <c r="E201" s="21" t="inlineStr">
@@ -19864,7 +19864,7 @@
       </c>
       <c r="D240" s="20" t="inlineStr">
         <is>
-          <t>*maa://30667 (78.63), maa://30666 (83.41), **maa://30739 (43.24), *maa://30723 (56.45), maa://39588 (88.68)</t>
+          <t>*maa://30667 (78.63), maa://30666 (83.41), **maa://30739 (43.24), *maa://30723 (56.45), maa://39588 (88.89)</t>
         </is>
       </c>
       <c r="E240" s="21" t="inlineStr">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="D249" s="20" t="inlineStr">
         <is>
-          <t>maa://42287 (90.48), maa://45570 (97.87), maa://42225 (100.0)</t>
+          <t>maa://42287 (90.48), maa://45570 (97.92), maa://42225 (100.0)</t>
         </is>
       </c>
       <c r="E249" s="21" t="inlineStr">
@@ -21322,7 +21322,7 @@
       </c>
       <c r="D267" s="20" t="inlineStr">
         <is>
-          <t>maa://49643 (86.36)</t>
+          <t>maa://49643 (86.96)</t>
         </is>
       </c>
       <c r="E267" s="21" t="inlineStr">
@@ -21592,7 +21592,7 @@
       </c>
       <c r="D272" s="20" t="inlineStr">
         <is>
-          <t>maa://51881 (99.16), maa://51630 (96.59), maa://56588 (94.12), *maa://55171 (57.14), maa://51893 (88.89)</t>
+          <t>maa://51881 (99.17), maa://51630 (96.59), maa://56588 (94.44), *maa://55171 (57.14), maa://51893 (88.89)</t>
         </is>
       </c>
       <c r="E272" s="21" t="inlineStr">
@@ -22510,7 +22510,7 @@
       </c>
       <c r="D289" s="20" t="inlineStr">
         <is>
-          <t>maa://30710 (97.87), maa://36845 (95.59), maa://31558 (97.06), **maa://39217 (41.18), maa://30668 (86.67)</t>
+          <t>maa://30710 (97.87), maa://36845 (95.62), maa://31558 (97.06), **maa://39217 (41.18), maa://30668 (86.67)</t>
         </is>
       </c>
       <c r="E289" s="21" t="inlineStr">
@@ -23266,7 +23266,7 @@
       </c>
       <c r="D303" s="20" t="inlineStr">
         <is>
-          <t>maa://50280 (97.52), maa://49642 (96.88), maa://49660 (92.86), *maa://50517 (80.0)</t>
+          <t>maa://50280 (97.54), maa://49642 (96.88), maa://49660 (92.86), *maa://50517 (80.0)</t>
         </is>
       </c>
       <c r="E303" s="21" t="inlineStr">
@@ -24238,7 +24238,7 @@
       </c>
       <c r="D321" s="20" t="inlineStr">
         <is>
-          <t>maa://39692 (99.61), maa://39810 (86.36)</t>
+          <t>maa://39692 (99.62), maa://39810 (86.36)</t>
         </is>
       </c>
       <c r="E321" s="21" t="inlineStr">
@@ -25912,7 +25912,7 @@
       </c>
       <c r="D352" s="17" t="inlineStr">
         <is>
-          <t>maa://49696 (99.55), maa://49695 (100.0), maa://49758 (98.44), *maa://52357 (71.43), *maa://59402 (66.67)</t>
+          <t>maa://49696 (99.55), maa://49695 (100.0), maa://49758 (98.44), *maa://52357 (71.43), *maa://59402 (71.43)</t>
         </is>
       </c>
       <c r="E352" s="17" t="inlineStr">
@@ -26128,7 +26128,7 @@
       </c>
       <c r="D356" s="17" t="inlineStr">
         <is>
-          <t>maa://36646 (98.79), maa://36845 (95.59), **maa://39217 (41.18), maa://51007 (98.15)</t>
+          <t>maa://36646 (98.79), maa://36845 (95.62), **maa://39217 (41.18), maa://51007 (98.15)</t>
         </is>
       </c>
       <c r="E356" s="17" t="inlineStr">
@@ -26398,7 +26398,7 @@
       </c>
       <c r="D361" s="17" t="inlineStr">
         <is>
-          <t>maa://40957 (93.36), maa://44635 (87.74), maa://48026 (96.39), maa://41035 (92.42), maa://44660 (92.31), maa://41128 (83.78)</t>
+          <t>maa://40957 (93.38), maa://44635 (87.74), maa://48026 (96.39), maa://41035 (92.42), maa://44660 (92.31), maa://41128 (83.78)</t>
         </is>
       </c>
       <c r="E361" s="17" t="inlineStr">
@@ -26992,7 +26992,7 @@
       </c>
       <c r="D372" s="17" t="inlineStr">
         <is>
-          <t>maa://44233 (92.16), maa://45570 (97.87)</t>
+          <t>maa://44233 (92.16), maa://45570 (97.92)</t>
         </is>
       </c>
       <c r="E372" s="17" t="inlineStr">
@@ -27262,7 +27262,7 @@
       </c>
       <c r="D377" s="17" t="inlineStr">
         <is>
-          <t>maa://42970 (83.86), maa://44745 (98.17), **maa://49516 (42.11), *maa://45952 (80.0), ***maa://46851 (14.29), *maa://44896 (77.78)</t>
+          <t>maa://42970 (83.53), maa://44745 (98.2), **maa://49516 (42.11), *maa://45952 (80.0), ***maa://46851 (14.29), *maa://44896 (77.78)</t>
         </is>
       </c>
       <c r="E377" s="17" t="inlineStr">
@@ -28018,7 +28018,7 @@
       </c>
       <c r="D391" s="17" t="inlineStr">
         <is>
-          <t>maa://51872 (96.65), maa://51876 (98.77), maa://51873 (100.0)</t>
+          <t>maa://51872 (96.7), maa://51876 (98.77), maa://51873 (100.0)</t>
         </is>
       </c>
       <c r="E391" s="17" t="inlineStr">
@@ -28072,7 +28072,7 @@
       </c>
       <c r="D392" s="17" t="inlineStr">
         <is>
-          <t>maa://59493 (96.3), maa://59603 (100.0)</t>
+          <t>maa://59493 (96.63), maa://59603 (100.0)</t>
         </is>
       </c>
       <c r="E392" s="17" t="inlineStr">

</xml_diff>